<commit_message>
updating link to OSR guidance
</commit_message>
<xml_diff>
--- a/docs/quality_questions_excel_template.xlsx
+++ b/docs/quality_questions_excel_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\coding_repositories\analysis_project_documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{276B85AB-C49F-49CE-AF0C-2CD09A945641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{70F91824-A8D7-4F32-BD07-685C02446ABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{4FDAA091-8849-4C6D-BF6B-DA0083E52E8E}"/>
   </bookViews>
@@ -2069,7 +2069,7 @@
 A record of validation and verification activities undertaken, outstanding tasks and remedial actions helps to confirm that the correct analysis has been performed for the required purpose and the chosen approach minimises risk.</t>
       </text>
     </comment>
-    <comment ref="D49" authorId="1" shapeId="0" xr:uid="{97D3B305-5D69-4B06-8A09-7E3DA165C2DF}">
+    <comment ref="D49" authorId="1" shapeId="0" xr:uid="{E64B8F05-593B-4703-8198-FA49CF19B366}">
       <text>
         <r>
           <rPr>
@@ -2079,8 +2079,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>T4.6: Hold regular reviews of the data management arrangements used and share best practice across the organisation to ensure data protection procedures remain effective. Keep pace with changing circumstances such as technological advances
-Q5.5: Periodically review the effectiveness of your processes and quality management approach and be open about findings and planned improvements</t>
+          <t>Q6.8: Collaborate with experts, other analysts and statistics producers in the UK and internationally where appropriate and share best practice</t>
         </r>
       </text>
     </comment>
@@ -2134,8 +2133,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>T4.6: Hold regular reviews of the data management arrangements used and share best practice across the organisation to ensure data protection procedures remain effective. Keep pace with changing circumstances such as technological advances
-Q5.5: Periodically review the effectiveness of your processes and quality management approach and be open about findings and planned improvements</t>
+          <t>Q6.8: Collaborate with experts, other analysts and statistics producers in the UK and internationally where appropriate and share best practice</t>
         </r>
       </text>
     </comment>
@@ -2245,13 +2243,14 @@
     </comment>
     <comment ref="M52" authorId="85" shapeId="0" xr:uid="{4ED4155D-4BE2-4D08-A20A-46CCE4600A2F}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     How do you assure yourselves that analysis carried out is correct?
 Reply:
     How do you ensure that input data are correct and in the expected structure and format?
-</t>
+Reply:
+    What do you feel is done well with regards to QA in your team? What could be better?</t>
       </text>
     </comment>
     <comment ref="C53" authorId="86" shapeId="0" xr:uid="{6E3DB2AC-3774-4582-BCA9-9EFF9F0AAE32}">
@@ -2708,7 +2707,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="243">
   <si>
     <t>This guidance is an ALPHA draft. It is in development and we are still working to ensure that it meets user needs.</t>
   </si>
@@ -3393,9 +3392,6 @@
   </si>
   <si>
     <t>V10.5</t>
-  </si>
-  <si>
-    <t>T4.6, Q5.5</t>
   </si>
   <si>
     <t>Q6.9, Q6.10</t>
@@ -4107,7 +4103,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -4347,9 +4343,6 @@
     <xf numFmtId="0" fontId="22" fillId="9" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -4398,16 +4391,16 @@
     <xf numFmtId="0" fontId="24" fillId="6" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5111,6 +5104,9 @@
     <text xml:space="preserve">How do you ensure that input data are correct and in the expected structure and format?
 </text>
   </threadedComment>
+  <threadedComment ref="M52" dT="2026-04-14T14:19:42.91" personId="{5DB4FC9B-6313-426F-8A60-5F9147BC1A6D}" id="{2C241690-7764-49AE-A917-F2C71B8C67AF}" parentId="{4ED4155D-4BE2-4D08-A20A-46CCE4600A2F}">
+    <text>What do you feel is done well with regards to QA in your team? What could be better?</text>
+  </threadedComment>
   <threadedComment ref="C53" dT="2024-09-02T09:23:29.30" personId="{D56F5C98-9DA8-4D6E-81A2-77932961FFC5}" id="{6E3DB2AC-3774-4582-BCA9-9EFF9F0AAE32}">
     <text>If you can, check that your outputs align with findings from previous runs of the analysis, alternate data sources, and comparable studies. This gives you confidence that the analysis works as expected. You should be able to explain any inconsistencies that you see.</text>
   </threadedComment>
@@ -5181,15 +5177,15 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" customWidth="1"/>
-    <col min="2" max="2" width="69.33203125" customWidth="1"/>
-    <col min="3" max="3" width="18.21875" customWidth="1"/>
-    <col min="4" max="4" width="13.88671875" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" customWidth="1"/>
+    <col min="2" max="2" width="69.36328125" customWidth="1"/>
+    <col min="3" max="3" width="18.1796875" customWidth="1"/>
+    <col min="4" max="4" width="13.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -5197,7 +5193,7 @@
       <c r="C1" s="2"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:4" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -5205,7 +5201,7 @@
       <c r="C2" s="2"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -5213,16 +5209,16 @@
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" ht="24.6" x14ac:dyDescent="0.4">
       <c r="A5" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>4</v>
       </c>
@@ -5236,25 +5232,25 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="104">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="103">
         <v>1.2</v>
       </c>
-      <c r="B8" s="104" t="s">
-        <v>240</v>
+      <c r="B8" s="103" t="s">
+        <v>239</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="103">
+      <c r="D8" s="102">
         <v>46048</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="85">
         <v>1.1000000000000001</v>
       </c>
-      <c r="B9" s="98" t="s">
+      <c r="B9" s="97" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="10" t="s">
@@ -5264,7 +5260,7 @@
         <v>45812</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>1</v>
       </c>
@@ -5278,31 +5274,31 @@
         <v>45601</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B11" s="6"/>
     </row>
-    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="13"/>
     </row>
-    <row r="14" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B15" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B16" s="6"/>
     </row>
-    <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
         <v>14</v>
       </c>
@@ -5310,7 +5306,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>16</v>
       </c>
@@ -5318,7 +5314,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>18</v>
       </c>
@@ -5326,7 +5322,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" ht="15.6" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>20</v>
       </c>
@@ -5334,7 +5330,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" ht="15.6" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>22</v>
       </c>
@@ -5342,11 +5338,11 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" ht="15.6" x14ac:dyDescent="0.25">
       <c r="A22" s="18"/>
       <c r="B22" s="19"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="20"/>
       <c r="B23" s="21"/>
     </row>
@@ -5367,23 +5363,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C48"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="104.44140625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="99.5546875" style="6" customWidth="1"/>
+    <col min="1" max="1" width="104.453125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="99.54296875" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
         <v>2</v>
       </c>
@@ -5393,218 +5389,218 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
         <v>25</v>
       </c>
       <c r="C5" s="26"/>
     </row>
-    <row r="6" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
         <v>26</v>
       </c>
       <c r="C6"/>
     </row>
-    <row r="7" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
         <v>27</v>
       </c>
       <c r="C7" s="26"/>
     </row>
-    <row r="8" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="28" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="29"/>
     </row>
-    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="30" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="31"/>
       <c r="C11" s="26"/>
     </row>
-    <row r="12" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="33"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="32"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="32" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="32" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="32" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="32" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="35" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="35" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="35" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="35" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="35" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="35" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="32" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="39.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="32" t="s">
         <v>42</v>
       </c>
       <c r="C25" s="26"/>
     </row>
-    <row r="26" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="35" t="s">
         <v>43</v>
       </c>
       <c r="C26" s="26"/>
     </row>
-    <row r="27" spans="1:3" ht="26.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="35" t="s">
         <v>44</v>
       </c>
       <c r="C27" s="26"/>
     </row>
-    <row r="28" spans="1:3" ht="26.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="41" t="s">
         <v>45</v>
       </c>
       <c r="C28" s="26"/>
     </row>
-    <row r="29" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="35" t="s">
         <v>46</v>
       </c>
       <c r="C29"/>
     </row>
-    <row r="30" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="36"/>
       <c r="C30" s="39"/>
     </row>
-    <row r="31" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="37" t="s">
         <v>47</v>
       </c>
       <c r="C31"/>
     </row>
-    <row r="32" spans="1:3" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="38"/>
       <c r="C32" s="26"/>
     </row>
-    <row r="33" spans="1:3" ht="78.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="25" t="s">
         <v>48</v>
       </c>
       <c r="C33"/>
     </row>
-    <row r="34" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="25"/>
       <c r="C34" s="26"/>
     </row>
-    <row r="35" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="25" t="s">
         <v>49</v>
       </c>
       <c r="C35"/>
     </row>
-    <row r="36" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="28" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="28" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="28" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="7.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" ht="7.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="25"/>
     </row>
-    <row r="40" spans="1:3" ht="29.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" ht="29.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="25" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="22.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="40" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="34"/>
     </row>
-    <row r="43" spans="1:3" ht="30" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="34" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="34"/>
     </row>
-    <row r="45" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="34" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="34"/>
     </row>
-    <row r="47" spans="1:3" ht="60" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A47" s="34" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="41" t="s">
         <v>58</v>
       </c>
@@ -5640,16 +5636,16 @@
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
   <dimension ref="A1:EZ38"/>
-  <sheetFormatPr defaultColWidth="7.109375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="7.08984375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.109375" style="44"/>
-    <col min="2" max="4" width="18.33203125" style="64" customWidth="1"/>
-    <col min="5" max="5" width="57.6640625" style="44" customWidth="1"/>
-    <col min="6" max="6" width="57.88671875" style="48" customWidth="1"/>
-    <col min="7" max="16384" width="7.109375" style="44"/>
+    <col min="1" max="1" width="7.08984375" style="44"/>
+    <col min="2" max="4" width="18.36328125" style="64" customWidth="1"/>
+    <col min="5" max="5" width="57.6328125" style="44" customWidth="1"/>
+    <col min="6" max="6" width="57.90625" style="48" customWidth="1"/>
+    <col min="7" max="16384" width="7.08984375" style="44"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:156" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:156" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="42" t="s">
         <v>24</v>
       </c>
@@ -5809,7 +5805,7 @@
       <c r="EY1" s="44"/>
       <c r="EZ1" s="44"/>
     </row>
-    <row r="2" spans="1:156" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:156" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="43"/>
       <c r="B2" s="43"/>
       <c r="C2" s="43"/>
@@ -5967,7 +5963,7 @@
       <c r="EY2" s="44"/>
       <c r="EZ2" s="44"/>
     </row>
-    <row r="3" spans="1:156" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:156" ht="24.6" x14ac:dyDescent="0.4">
       <c r="A3" s="45" t="s">
         <v>59</v>
       </c>
@@ -5978,96 +5974,96 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:156" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:156" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="47" t="s">
         <v>61</v>
       </c>
-      <c r="C4" s="109"/>
-      <c r="D4" s="110"/>
-      <c r="E4" s="111"/>
-    </row>
-    <row r="5" spans="1:156" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C4" s="105"/>
+      <c r="D4" s="106"/>
+      <c r="E4" s="107"/>
+    </row>
+    <row r="5" spans="1:156" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="109"/>
-      <c r="D5" s="110"/>
-      <c r="E5" s="111"/>
-    </row>
-    <row r="6" spans="1:156" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C5" s="105"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="107"/>
+    </row>
+    <row r="6" spans="1:156" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="49" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="109"/>
-      <c r="D6" s="110"/>
-      <c r="E6" s="111"/>
+      <c r="C6" s="105"/>
+      <c r="D6" s="106"/>
+      <c r="E6" s="107"/>
       <c r="F6" s="48" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:156" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:156" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="49" t="s">
         <v>65</v>
       </c>
-      <c r="C7" s="109"/>
-      <c r="D7" s="110"/>
-      <c r="E7" s="111"/>
+      <c r="C7" s="105"/>
+      <c r="D7" s="106"/>
+      <c r="E7" s="107"/>
       <c r="F7" s="48" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="8" spans="1:156" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:156" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="49" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="109"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
-    </row>
-    <row r="9" spans="1:156" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C8" s="105"/>
+      <c r="D8" s="106"/>
+      <c r="E8" s="107"/>
+    </row>
+    <row r="9" spans="1:156" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="109"/>
-      <c r="D9" s="110"/>
-      <c r="E9" s="111"/>
+      <c r="C9" s="105"/>
+      <c r="D9" s="106"/>
+      <c r="E9" s="107"/>
       <c r="F9" s="48" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="10" spans="1:156" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:156" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="49" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="109"/>
-      <c r="D10" s="110"/>
-      <c r="E10" s="111"/>
-    </row>
-    <row r="11" spans="1:156" ht="45" x14ac:dyDescent="0.2">
+      <c r="C10" s="105"/>
+      <c r="D10" s="106"/>
+      <c r="E10" s="107"/>
+    </row>
+    <row r="11" spans="1:156" ht="45" x14ac:dyDescent="0.25">
       <c r="B11" s="49" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="109"/>
-      <c r="D11" s="110"/>
-      <c r="E11" s="111"/>
+      <c r="C11" s="105"/>
+      <c r="D11" s="106"/>
+      <c r="E11" s="107"/>
       <c r="F11" s="48" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:156" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:156" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="50" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="109"/>
-      <c r="D12" s="110"/>
-      <c r="E12" s="111"/>
-    </row>
-    <row r="13" spans="1:156" x14ac:dyDescent="0.2">
+      <c r="C12" s="105"/>
+      <c r="D12" s="106"/>
+      <c r="E12" s="107"/>
+    </row>
+    <row r="13" spans="1:156" x14ac:dyDescent="0.25">
       <c r="B13" s="43"/>
       <c r="C13" s="43"/>
       <c r="D13" s="43"/>
     </row>
-    <row r="14" spans="1:156" ht="48" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:156" ht="46.8" x14ac:dyDescent="0.4">
       <c r="A14" s="45" t="s">
         <v>74</v>
       </c>
@@ -6078,77 +6074,77 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:156" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:156" ht="24.6" x14ac:dyDescent="0.4">
       <c r="A15" s="45"/>
       <c r="B15" s="51"/>
       <c r="C15" s="51" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="112" t="s">
+      <c r="D15" s="111" t="s">
         <v>77</v>
       </c>
-      <c r="E15" s="113"/>
+      <c r="E15" s="112"/>
       <c r="F15" s="52" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:156" ht="63" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:156" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="53" t="s">
         <v>193</v>
       </c>
       <c r="C16" s="54"/>
-      <c r="D16" s="114"/>
-      <c r="E16" s="115"/>
+      <c r="D16" s="113"/>
+      <c r="E16" s="114"/>
       <c r="F16" s="48" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="78" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="78" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="50" t="s">
         <v>80</v>
       </c>
       <c r="C17" s="55"/>
-      <c r="D17" s="109"/>
-      <c r="E17" s="111"/>
-    </row>
-    <row r="18" spans="1:6" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D17" s="105"/>
+      <c r="E17" s="107"/>
+    </row>
+    <row r="18" spans="1:6" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="56" t="s">
         <v>194</v>
       </c>
       <c r="C18" s="57"/>
-      <c r="D18" s="109"/>
-      <c r="E18" s="111"/>
+      <c r="D18" s="105"/>
+      <c r="E18" s="107"/>
       <c r="F18" s="48" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="56" t="s">
         <v>82</v>
       </c>
       <c r="C19" s="57"/>
-      <c r="D19" s="109"/>
-      <c r="E19" s="111"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="107"/>
       <c r="F19" s="48" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B20" s="43"/>
       <c r="C20" s="43"/>
       <c r="D20" s="43"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B21" s="43"/>
       <c r="C21" s="43"/>
       <c r="D21" s="43"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B22" s="43"/>
       <c r="C22" s="43"/>
       <c r="D22" s="43"/>
     </row>
-    <row r="23" spans="1:6" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" ht="24.6" x14ac:dyDescent="0.4">
       <c r="A23" s="45" t="s">
         <v>83</v>
       </c>
@@ -6156,44 +6152,44 @@
       <c r="C23" s="43"/>
       <c r="D23" s="43"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B24" s="43"/>
       <c r="C24" s="43"/>
       <c r="D24" s="43"/>
     </row>
-    <row r="25" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="58" t="s">
         <v>84</v>
       </c>
-      <c r="C25" s="106"/>
-      <c r="D25" s="116"/>
+      <c r="C25" s="108"/>
+      <c r="D25" s="115"/>
       <c r="E25" s="59"/>
     </row>
-    <row r="26" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="58" t="s">
         <v>85</v>
       </c>
-      <c r="C26" s="106"/>
-      <c r="D26" s="107"/>
-      <c r="E26" s="108"/>
-    </row>
-    <row r="27" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C26" s="108"/>
+      <c r="D26" s="109"/>
+      <c r="E26" s="110"/>
+    </row>
+    <row r="27" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="58" t="s">
         <v>86</v>
       </c>
-      <c r="C27" s="106"/>
-      <c r="D27" s="107"/>
-      <c r="E27" s="108"/>
-    </row>
-    <row r="28" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C27" s="108"/>
+      <c r="D27" s="109"/>
+      <c r="E27" s="110"/>
+    </row>
+    <row r="28" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="58" t="s">
         <v>87</v>
       </c>
-      <c r="C28" s="106"/>
-      <c r="D28" s="107"/>
-      <c r="E28" s="108"/>
-    </row>
-    <row r="32" spans="1:6" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="C28" s="108"/>
+      <c r="D28" s="109"/>
+      <c r="E28" s="110"/>
+    </row>
+    <row r="32" spans="1:6" ht="24.6" x14ac:dyDescent="0.4">
       <c r="A32" s="45" t="s">
         <v>88</v>
       </c>
@@ -6201,7 +6197,7 @@
       <c r="C32" s="43"/>
       <c r="D32" s="43"/>
     </row>
-    <row r="33" spans="1:6" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" ht="24.6" x14ac:dyDescent="0.4">
       <c r="A33" s="45"/>
       <c r="B33" s="51"/>
       <c r="C33" s="51" t="s">
@@ -6217,7 +6213,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" ht="15.6" x14ac:dyDescent="0.25">
       <c r="B34" s="53" t="s">
         <v>90</v>
       </c>
@@ -6225,23 +6221,23 @@
       <c r="D34" s="54"/>
       <c r="E34" s="61"/>
     </row>
-    <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" ht="15.6" x14ac:dyDescent="0.25">
       <c r="B35" s="50" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C35" s="55"/>
       <c r="D35" s="55"/>
       <c r="E35" s="62"/>
     </row>
-    <row r="36" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" ht="15.6" x14ac:dyDescent="0.25">
       <c r="B36" s="56" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C36" s="57"/>
       <c r="D36" s="57"/>
       <c r="E36" s="63"/>
     </row>
-    <row r="37" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" ht="15.6" x14ac:dyDescent="0.25">
       <c r="B37" s="56" t="s">
         <v>91</v>
       </c>
@@ -6249,19 +6245,13 @@
       <c r="D37" s="57"/>
       <c r="E37" s="63"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B38" s="43"/>
       <c r="C38" s="43"/>
       <c r="D38" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="C8:E8"/>
     <mergeCell ref="C28:E28"/>
     <mergeCell ref="C10:E10"/>
     <mergeCell ref="C11:E11"/>
@@ -6274,6 +6264,12 @@
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="C26:E26"/>
     <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="C8:E8"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F15" r:id="rId1" display="Quality Questions" xr:uid="{1DBDD650-1A86-4D83-84AD-FB97A897BCC1}"/>
@@ -6290,38 +6286,38 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U73"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="6.33203125" style="81" customWidth="1"/>
-    <col min="3" max="3" width="58.21875" style="83" customWidth="1"/>
-    <col min="4" max="4" width="12.77734375" style="97" customWidth="1"/>
-    <col min="5" max="5" width="22.77734375" style="81" customWidth="1"/>
-    <col min="6" max="6" width="88.109375" style="97" customWidth="1"/>
-    <col min="7" max="9" width="24.21875" style="81" customWidth="1"/>
-    <col min="10" max="10" width="28.44140625" style="81" customWidth="1"/>
-    <col min="11" max="11" width="51.88671875" style="81" customWidth="1"/>
-    <col min="12" max="12" width="29.21875" style="79" customWidth="1"/>
-    <col min="13" max="13" width="16.77734375" style="79" customWidth="1"/>
-    <col min="14" max="14" width="23.6640625" customWidth="1"/>
-    <col min="15" max="15" width="20.109375" customWidth="1"/>
-    <col min="16" max="16" width="22.44140625" customWidth="1"/>
-    <col min="17" max="17" width="22.88671875" customWidth="1"/>
-    <col min="18" max="18" width="23.5546875" customWidth="1"/>
-    <col min="19" max="19" width="26.6640625" customWidth="1"/>
-    <col min="20" max="20" width="21.6640625" customWidth="1"/>
+    <col min="2" max="2" width="6.36328125" style="81" customWidth="1"/>
+    <col min="3" max="3" width="58.1796875" style="83" customWidth="1"/>
+    <col min="4" max="4" width="12.81640625" style="96" customWidth="1"/>
+    <col min="5" max="5" width="22.81640625" style="81" customWidth="1"/>
+    <col min="6" max="6" width="88.08984375" style="96" customWidth="1"/>
+    <col min="7" max="9" width="24.1796875" style="81" customWidth="1"/>
+    <col min="10" max="10" width="28.453125" style="81" customWidth="1"/>
+    <col min="11" max="11" width="51.90625" style="81" customWidth="1"/>
+    <col min="12" max="12" width="29.1796875" style="79" customWidth="1"/>
+    <col min="13" max="13" width="16.81640625" style="79" customWidth="1"/>
+    <col min="14" max="14" width="23.6328125" customWidth="1"/>
+    <col min="15" max="15" width="20.08984375" customWidth="1"/>
+    <col min="16" max="16" width="22.453125" customWidth="1"/>
+    <col min="17" max="17" width="22.90625" customWidth="1"/>
+    <col min="18" max="18" width="23.54296875" customWidth="1"/>
+    <col min="19" max="19" width="26.6328125" customWidth="1"/>
+    <col min="20" max="20" width="21.6328125" customWidth="1"/>
     <col min="21" max="21" width="18" customWidth="1"/>
-    <col min="22" max="22" width="24.5546875" customWidth="1"/>
+    <col min="22" max="22" width="24.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="65" customFormat="1" ht="126.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="118" t="s">
+    <row r="1" spans="1:21" s="65" customFormat="1" ht="126.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="117" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="118"/>
-      <c r="C1" s="118"/>
-      <c r="D1" s="118"/>
-      <c r="E1" s="118"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
       <c r="F1" s="43"/>
       <c r="G1" s="43"/>
       <c r="H1" s="43"/>
@@ -6330,19 +6326,19 @@
       <c r="K1" s="43"/>
       <c r="L1" s="43"/>
       <c r="M1" s="43"/>
-      <c r="N1" s="119" t="s">
+      <c r="N1" s="118" t="s">
         <v>93</v>
       </c>
-      <c r="O1" s="120"/>
-      <c r="P1" s="120"/>
-      <c r="Q1" s="120"/>
-      <c r="R1" s="120"/>
-      <c r="S1" s="120"/>
-      <c r="T1" s="120"/>
-      <c r="U1" s="121"/>
-    </row>
-    <row r="2" spans="1:21" s="66" customFormat="1" ht="93" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="105" t="s">
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="120"/>
+    </row>
+    <row r="2" spans="1:21" s="66" customFormat="1" ht="93" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="104" t="s">
         <v>94</v>
       </c>
       <c r="B2" s="86" t="s">
@@ -6351,10 +6347,10 @@
       <c r="C2" s="86" t="s">
         <v>96</v>
       </c>
-      <c r="D2" s="105" t="s">
+      <c r="D2" s="104" t="s">
         <v>97</v>
       </c>
-      <c r="E2" s="105" t="s">
+      <c r="E2" s="104" t="s">
         <v>98</v>
       </c>
       <c r="F2" s="87" t="s">
@@ -6378,48 +6374,48 @@
       <c r="L2" s="88" t="s">
         <v>105</v>
       </c>
-      <c r="M2" s="89" t="s">
+      <c r="M2" s="88" t="s">
         <v>106</v>
       </c>
-      <c r="N2" s="90" t="s">
+      <c r="N2" s="89" t="s">
         <v>107</v>
       </c>
-      <c r="O2" s="90" t="s">
+      <c r="O2" s="89" t="s">
         <v>108</v>
       </c>
-      <c r="P2" s="90" t="s">
+      <c r="P2" s="89" t="s">
         <v>109</v>
       </c>
-      <c r="Q2" s="90" t="s">
+      <c r="Q2" s="89" t="s">
         <v>110</v>
       </c>
-      <c r="R2" s="90" t="s">
+      <c r="R2" s="89" t="s">
         <v>111</v>
       </c>
-      <c r="S2" s="90" t="s">
+      <c r="S2" s="89" t="s">
         <v>112</v>
       </c>
-      <c r="T2" s="90" t="s">
+      <c r="T2" s="89" t="s">
         <v>113</v>
       </c>
-      <c r="U2" s="90" t="s">
+      <c r="U2" s="89" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="122" t="s">
+    <row r="3" spans="1:21" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="121" t="s">
         <v>191</v>
       </c>
-      <c r="B3" s="91">
-        <v>1</v>
-      </c>
-      <c r="C3" s="99" t="s">
+      <c r="B3" s="90">
+        <v>1</v>
+      </c>
+      <c r="C3" s="98" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="92" t="s">
+      <c r="D3" s="91" t="s">
         <v>195</v>
       </c>
-      <c r="E3" s="92" t="s">
+      <c r="E3" s="91" t="s">
         <v>184</v>
       </c>
       <c r="F3" s="67"/>
@@ -6459,19 +6455,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="122"/>
-      <c r="B4" s="92">
+    <row r="4" spans="1:21" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="121"/>
+      <c r="B4" s="91">
         <f>B3+1</f>
         <v>2</v>
       </c>
-      <c r="C4" s="99" t="s">
+      <c r="C4" s="98" t="s">
         <v>117</v>
       </c>
-      <c r="D4" s="92" t="s">
+      <c r="D4" s="91" t="s">
         <v>195</v>
       </c>
-      <c r="E4" s="92" t="s">
+      <c r="E4" s="91" t="s">
         <v>184</v>
       </c>
       <c r="F4" s="68"/>
@@ -6509,19 +6505,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="122"/>
-      <c r="B5" s="92">
+    <row r="5" spans="1:21" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="121"/>
+      <c r="B5" s="91">
         <f t="shared" ref="B5:B21" si="0">B4+1</f>
         <v>3</v>
       </c>
-      <c r="C5" s="99" t="s">
+      <c r="C5" s="98" t="s">
         <v>118</v>
       </c>
-      <c r="D5" s="92" t="s">
+      <c r="D5" s="91" t="s">
         <v>196</v>
       </c>
-      <c r="E5" s="92" t="s">
+      <c r="E5" s="91" t="s">
         <v>90</v>
       </c>
       <c r="F5" s="68"/>
@@ -6557,20 +6553,20 @@
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="18.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="122"/>
-      <c r="B6" s="92">
+    <row r="6" spans="1:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="121"/>
+      <c r="B6" s="91">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="99" t="s">
+      <c r="C6" s="98" t="s">
         <v>119</v>
       </c>
-      <c r="D6" s="92" t="s">
+      <c r="D6" s="91" t="s">
         <v>197</v>
       </c>
-      <c r="E6" s="92" t="s">
-        <v>241</v>
+      <c r="E6" s="91" t="s">
+        <v>240</v>
       </c>
       <c r="F6" s="68"/>
       <c r="G6" s="68"/>
@@ -6605,19 +6601,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="122"/>
-      <c r="B7" s="92">
+    <row r="7" spans="1:21" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="121"/>
+      <c r="B7" s="91">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C7" s="99" t="s">
+      <c r="C7" s="98" t="s">
         <v>120</v>
       </c>
-      <c r="D7" s="92" t="s">
+      <c r="D7" s="91" t="s">
         <v>195</v>
       </c>
-      <c r="E7" s="92" t="s">
+      <c r="E7" s="91" t="s">
         <v>184</v>
       </c>
       <c r="F7" s="68"/>
@@ -6655,19 +6651,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="122"/>
-      <c r="B8" s="92">
+    <row r="8" spans="1:21" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="121"/>
+      <c r="B8" s="91">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C8" s="99" t="s">
+      <c r="C8" s="98" t="s">
         <v>121</v>
       </c>
-      <c r="D8" s="92" t="s">
+      <c r="D8" s="91" t="s">
         <v>198</v>
       </c>
-      <c r="E8" s="92" t="s">
+      <c r="E8" s="91" t="s">
         <v>159</v>
       </c>
       <c r="F8" s="68"/>
@@ -6703,19 +6699,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="18.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="122"/>
-      <c r="B9" s="92">
+    <row r="9" spans="1:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="121"/>
+      <c r="B9" s="91">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C9" s="99" t="s">
+      <c r="C9" s="98" t="s">
         <v>122</v>
       </c>
-      <c r="D9" s="92" t="s">
+      <c r="D9" s="91" t="s">
         <v>199</v>
       </c>
-      <c r="E9" s="92" t="s">
+      <c r="E9" s="91" t="s">
         <v>138</v>
       </c>
       <c r="F9" s="68"/>
@@ -6753,20 +6749,20 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="122"/>
-      <c r="B10" s="92">
+    <row r="10" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="121"/>
+      <c r="B10" s="91">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C10" s="99" t="s">
+      <c r="C10" s="98" t="s">
         <v>123</v>
       </c>
-      <c r="D10" s="92" t="s">
+      <c r="D10" s="91" t="s">
         <v>200</v>
       </c>
-      <c r="E10" s="92" t="s">
-        <v>242</v>
+      <c r="E10" s="91" t="s">
+        <v>241</v>
       </c>
       <c r="F10" s="68"/>
       <c r="G10" s="68"/>
@@ -6803,19 +6799,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="122"/>
-      <c r="B11" s="92">
+    <row r="11" spans="1:21" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="121"/>
+      <c r="B11" s="91">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C11" s="99" t="s">
+      <c r="C11" s="98" t="s">
         <v>124</v>
       </c>
-      <c r="D11" s="92" t="s">
+      <c r="D11" s="91" t="s">
         <v>196</v>
       </c>
-      <c r="E11" s="92" t="s">
+      <c r="E11" s="91" t="s">
         <v>90</v>
       </c>
       <c r="F11" s="68"/>
@@ -6851,19 +6847,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="18.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="122"/>
-      <c r="B12" s="92">
+    <row r="12" spans="1:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="121"/>
+      <c r="B12" s="91">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C12" s="99" t="s">
+      <c r="C12" s="98" t="s">
         <v>125</v>
       </c>
-      <c r="D12" s="92" t="s">
+      <c r="D12" s="91" t="s">
         <v>201</v>
       </c>
-      <c r="E12" s="92" t="s">
+      <c r="E12" s="91" t="s">
         <v>138</v>
       </c>
       <c r="F12" s="68"/>
@@ -6899,19 +6895,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="122"/>
-      <c r="B13" s="92">
+    <row r="13" spans="1:21" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="121"/>
+      <c r="B13" s="91">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C13" s="99" t="s">
+      <c r="C13" s="98" t="s">
         <v>190</v>
       </c>
-      <c r="D13" s="92" t="s">
+      <c r="D13" s="91" t="s">
         <v>202</v>
       </c>
-      <c r="E13" s="92" t="s">
+      <c r="E13" s="91" t="s">
         <v>90</v>
       </c>
       <c r="F13" s="68"/>
@@ -6947,19 +6943,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="122"/>
-      <c r="B14" s="92">
+    <row r="14" spans="1:21" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="121"/>
+      <c r="B14" s="91">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C14" s="99" t="s">
+      <c r="C14" s="98" t="s">
         <v>126</v>
       </c>
-      <c r="D14" s="92" t="s">
+      <c r="D14" s="91" t="s">
         <v>203</v>
       </c>
-      <c r="E14" s="92" t="s">
+      <c r="E14" s="91" t="s">
         <v>90</v>
       </c>
       <c r="F14" s="68"/>
@@ -6997,19 +6993,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="122"/>
-      <c r="B15" s="92">
+    <row r="15" spans="1:21" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="121"/>
+      <c r="B15" s="91">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C15" s="99" t="s">
+      <c r="C15" s="98" t="s">
         <v>127</v>
       </c>
-      <c r="D15" s="92" t="s">
+      <c r="D15" s="91" t="s">
         <v>203</v>
       </c>
-      <c r="E15" s="92" t="s">
+      <c r="E15" s="91" t="s">
         <v>90</v>
       </c>
       <c r="F15" s="68"/>
@@ -7045,20 +7041,20 @@
         <v>116</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="122"/>
-      <c r="B16" s="92">
+    <row r="16" spans="1:21" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="121"/>
+      <c r="B16" s="91">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C16" s="99" t="s">
+      <c r="C16" s="98" t="s">
         <v>128</v>
       </c>
-      <c r="D16" s="92" t="s">
+      <c r="D16" s="91" t="s">
         <v>204</v>
       </c>
-      <c r="E16" s="92" t="s">
-        <v>243</v>
+      <c r="E16" s="91" t="s">
+        <v>242</v>
       </c>
       <c r="F16" s="68"/>
       <c r="G16" s="68"/>
@@ -7095,19 +7091,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="17" spans="1:21" ht="37.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="122"/>
-      <c r="B17" s="92">
+    <row r="17" spans="1:21" ht="37.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="121"/>
+      <c r="B17" s="91">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C17" s="99" t="s">
+      <c r="C17" s="98" t="s">
         <v>129</v>
       </c>
-      <c r="D17" s="92" t="s">
+      <c r="D17" s="91" t="s">
         <v>205</v>
       </c>
-      <c r="E17" s="92" t="s">
+      <c r="E17" s="91" t="s">
         <v>187</v>
       </c>
       <c r="F17" s="68"/>
@@ -7143,19 +7139,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="18" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="122"/>
-      <c r="B18" s="92">
+    <row r="18" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="121"/>
+      <c r="B18" s="91">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C18" s="99" t="s">
+      <c r="C18" s="98" t="s">
         <v>130</v>
       </c>
-      <c r="D18" s="92" t="s">
+      <c r="D18" s="91" t="s">
         <v>206</v>
       </c>
-      <c r="E18" s="92" t="s">
+      <c r="E18" s="91" t="s">
         <v>181</v>
       </c>
       <c r="F18" s="68"/>
@@ -7191,19 +7187,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="38.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="122"/>
-      <c r="B19" s="92">
+    <row r="19" spans="1:21" ht="38.700000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="121"/>
+      <c r="B19" s="91">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C19" s="99" t="s">
+      <c r="C19" s="98" t="s">
         <v>131</v>
       </c>
-      <c r="D19" s="92" t="s">
+      <c r="D19" s="91" t="s">
         <v>207</v>
       </c>
-      <c r="E19" s="92" t="s">
+      <c r="E19" s="91" t="s">
         <v>138</v>
       </c>
       <c r="F19" s="68"/>
@@ -7239,20 +7235,20 @@
         <v>116</v>
       </c>
     </row>
-    <row r="20" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="122"/>
-      <c r="B20" s="92">
+    <row r="20" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="121"/>
+      <c r="B20" s="91">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C20" s="99" t="s">
+      <c r="C20" s="98" t="s">
         <v>132</v>
       </c>
-      <c r="D20" s="92" t="s">
+      <c r="D20" s="91" t="s">
         <v>208</v>
       </c>
-      <c r="E20" s="92" t="s">
-        <v>243</v>
+      <c r="E20" s="91" t="s">
+        <v>242</v>
       </c>
       <c r="F20" s="68"/>
       <c r="G20" s="68"/>
@@ -7287,20 +7283,20 @@
         <v>116</v>
       </c>
     </row>
-    <row r="21" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="122"/>
-      <c r="B21" s="92">
+    <row r="21" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="121"/>
+      <c r="B21" s="91">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C21" s="99" t="s">
+      <c r="C21" s="98" t="s">
         <v>133</v>
       </c>
-      <c r="D21" s="92" t="s">
+      <c r="D21" s="91" t="s">
         <v>209</v>
       </c>
-      <c r="E21" s="92" t="s">
-        <v>243</v>
+      <c r="E21" s="91" t="s">
+        <v>242</v>
       </c>
       <c r="F21" s="68"/>
       <c r="G21" s="68"/>
@@ -7337,21 +7333,21 @@
         <v>116</v>
       </c>
     </row>
-    <row r="22" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="123" t="s">
+    <row r="22" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="122" t="s">
         <v>134</v>
       </c>
-      <c r="B22" s="93">
+      <c r="B22" s="92">
         <f>B21+1</f>
         <v>20</v>
       </c>
-      <c r="C22" s="100" t="s">
+      <c r="C22" s="99" t="s">
         <v>135</v>
       </c>
-      <c r="D22" s="93" t="s">
+      <c r="D22" s="92" t="s">
         <v>210</v>
       </c>
-      <c r="E22" s="93" t="s">
+      <c r="E22" s="92" t="s">
         <v>182</v>
       </c>
       <c r="F22" s="73"/>
@@ -7387,19 +7383,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="123"/>
-      <c r="B23" s="93">
+    <row r="23" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="122"/>
+      <c r="B23" s="92">
         <f t="shared" ref="B23:B27" si="1">B22+1</f>
         <v>21</v>
       </c>
-      <c r="C23" s="100" t="s">
+      <c r="C23" s="99" t="s">
         <v>136</v>
       </c>
-      <c r="D23" s="93" t="s">
+      <c r="D23" s="92" t="s">
         <v>211</v>
       </c>
-      <c r="E23" s="93" t="s">
+      <c r="E23" s="92" t="s">
         <v>182</v>
       </c>
       <c r="F23" s="73"/>
@@ -7439,19 +7435,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="123"/>
-      <c r="B24" s="93">
+    <row r="24" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="122"/>
+      <c r="B24" s="92">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="C24" s="100" t="s">
+      <c r="C24" s="99" t="s">
         <v>137</v>
       </c>
-      <c r="D24" s="93" t="s">
+      <c r="D24" s="92" t="s">
         <v>212</v>
       </c>
-      <c r="E24" s="93" t="s">
+      <c r="E24" s="92" t="s">
         <v>138</v>
       </c>
       <c r="F24" s="73"/>
@@ -7489,19 +7485,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="25" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="123"/>
-      <c r="B25" s="93">
+    <row r="25" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="122"/>
+      <c r="B25" s="92">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
-      <c r="C25" s="100" t="s">
+      <c r="C25" s="99" t="s">
         <v>139</v>
       </c>
-      <c r="D25" s="93" t="s">
+      <c r="D25" s="92" t="s">
         <v>213</v>
       </c>
-      <c r="E25" s="93" t="s">
+      <c r="E25" s="92" t="s">
         <v>138</v>
       </c>
       <c r="F25" s="73"/>
@@ -7539,19 +7535,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="26" spans="1:21" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="123"/>
-      <c r="B26" s="93">
+    <row r="26" spans="1:21" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="122"/>
+      <c r="B26" s="92">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="C26" s="100" t="s">
+      <c r="C26" s="99" t="s">
         <v>140</v>
       </c>
-      <c r="D26" s="93" t="s">
+      <c r="D26" s="92" t="s">
         <v>214</v>
       </c>
-      <c r="E26" s="93" t="s">
+      <c r="E26" s="92" t="s">
         <v>182</v>
       </c>
       <c r="F26" s="73"/>
@@ -7591,19 +7587,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:21" ht="18.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="123"/>
-      <c r="B27" s="93">
+    <row r="27" spans="1:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="122"/>
+      <c r="B27" s="92">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="C27" s="100" t="s">
+      <c r="C27" s="99" t="s">
         <v>141</v>
       </c>
-      <c r="D27" s="93" t="s">
+      <c r="D27" s="92" t="s">
         <v>215</v>
       </c>
-      <c r="E27" s="93" t="s">
+      <c r="E27" s="92" t="s">
         <v>138</v>
       </c>
       <c r="F27" s="73"/>
@@ -7641,21 +7637,21 @@
         <v>116</v>
       </c>
     </row>
-    <row r="28" spans="1:21" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="124" t="s">
+    <row r="28" spans="1:21" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="123" t="s">
         <v>192</v>
       </c>
-      <c r="B28" s="94">
+      <c r="B28" s="93">
         <f>B27+1</f>
         <v>26</v>
       </c>
-      <c r="C28" s="101" t="s">
+      <c r="C28" s="100" t="s">
         <v>142</v>
       </c>
-      <c r="D28" s="94" t="s">
+      <c r="D28" s="93" t="s">
         <v>216</v>
       </c>
-      <c r="E28" s="94" t="s">
+      <c r="E28" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F28" s="84"/>
@@ -7691,19 +7687,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="29" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="124"/>
-      <c r="B29" s="94">
+    <row r="29" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="123"/>
+      <c r="B29" s="93">
         <f t="shared" ref="B29:B54" si="2">B28+1</f>
         <v>27</v>
       </c>
-      <c r="C29" s="101" t="s">
+      <c r="C29" s="100" t="s">
         <v>143</v>
       </c>
-      <c r="D29" s="94" t="s">
+      <c r="D29" s="93" t="s">
         <v>217</v>
       </c>
-      <c r="E29" s="94" t="s">
+      <c r="E29" s="93" t="s">
         <v>183</v>
       </c>
       <c r="F29" s="84"/>
@@ -7739,19 +7735,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="30" spans="1:21" ht="18.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="124"/>
-      <c r="B30" s="94">
+    <row r="30" spans="1:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="123"/>
+      <c r="B30" s="93">
         <f t="shared" si="2"/>
         <v>28</v>
       </c>
-      <c r="C30" s="101" t="s">
+      <c r="C30" s="100" t="s">
         <v>144</v>
       </c>
-      <c r="D30" s="94" t="s">
+      <c r="D30" s="93" t="s">
         <v>218</v>
       </c>
-      <c r="E30" s="94" t="s">
+      <c r="E30" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F30" s="84"/>
@@ -7789,19 +7785,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="31" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="124"/>
-      <c r="B31" s="94">
+    <row r="31" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="123"/>
+      <c r="B31" s="93">
         <f t="shared" si="2"/>
         <v>29</v>
       </c>
-      <c r="C31" s="101" t="s">
+      <c r="C31" s="100" t="s">
         <v>145</v>
       </c>
-      <c r="D31" s="94" t="s">
+      <c r="D31" s="93" t="s">
         <v>219</v>
       </c>
-      <c r="E31" s="94" t="s">
+      <c r="E31" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F31" s="84"/>
@@ -7839,19 +7835,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="124"/>
-      <c r="B32" s="94">
+    <row r="32" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="123"/>
+      <c r="B32" s="93">
         <f t="shared" si="2"/>
         <v>30</v>
       </c>
-      <c r="C32" s="101" t="s">
+      <c r="C32" s="100" t="s">
         <v>146</v>
       </c>
-      <c r="D32" s="94" t="s">
+      <c r="D32" s="93" t="s">
         <v>220</v>
       </c>
-      <c r="E32" s="94" t="s">
+      <c r="E32" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F32" s="84"/>
@@ -7887,19 +7883,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="33" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="124"/>
-      <c r="B33" s="94">
+    <row r="33" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="123"/>
+      <c r="B33" s="93">
         <f t="shared" si="2"/>
         <v>31</v>
       </c>
-      <c r="C33" s="101" t="s">
+      <c r="C33" s="100" t="s">
         <v>147</v>
       </c>
-      <c r="D33" s="94" t="s">
+      <c r="D33" s="93" t="s">
         <v>219</v>
       </c>
-      <c r="E33" s="94" t="s">
+      <c r="E33" s="93" t="s">
         <v>184</v>
       </c>
       <c r="F33" s="84"/>
@@ -7937,19 +7933,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="34" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="124"/>
-      <c r="B34" s="94">
+    <row r="34" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="123"/>
+      <c r="B34" s="93">
         <f t="shared" si="2"/>
         <v>32</v>
       </c>
-      <c r="C34" s="101" t="s">
+      <c r="C34" s="100" t="s">
         <v>148</v>
       </c>
-      <c r="D34" s="94" t="s">
+      <c r="D34" s="93" t="s">
         <v>219</v>
       </c>
-      <c r="E34" s="94" t="s">
+      <c r="E34" s="93" t="s">
         <v>149</v>
       </c>
       <c r="F34" s="84"/>
@@ -7987,19 +7983,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="35" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="124"/>
-      <c r="B35" s="94">
+    <row r="35" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="123"/>
+      <c r="B35" s="93">
         <f t="shared" si="2"/>
         <v>33</v>
       </c>
-      <c r="C35" s="101" t="s">
+      <c r="C35" s="100" t="s">
         <v>150</v>
       </c>
-      <c r="D35" s="94" t="s">
+      <c r="D35" s="93" t="s">
         <v>219</v>
       </c>
-      <c r="E35" s="94" t="s">
+      <c r="E35" s="93" t="s">
         <v>184</v>
       </c>
       <c r="F35" s="84"/>
@@ -8037,19 +8033,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="36" spans="1:21" ht="45.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="124"/>
-      <c r="B36" s="94">
+    <row r="36" spans="1:21" ht="45.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="123"/>
+      <c r="B36" s="93">
         <f t="shared" si="2"/>
         <v>34</v>
       </c>
-      <c r="C36" s="101" t="s">
+      <c r="C36" s="100" t="s">
         <v>151</v>
       </c>
-      <c r="D36" s="94" t="s">
+      <c r="D36" s="93" t="s">
         <v>220</v>
       </c>
-      <c r="E36" s="94" t="s">
+      <c r="E36" s="93" t="s">
         <v>184</v>
       </c>
       <c r="F36" s="84"/>
@@ -8087,19 +8083,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="37" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="125"/>
-      <c r="B37" s="94">
+    <row r="37" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="124"/>
+      <c r="B37" s="93">
         <f t="shared" si="2"/>
         <v>35</v>
       </c>
-      <c r="C37" s="101" t="s">
+      <c r="C37" s="100" t="s">
         <v>152</v>
       </c>
-      <c r="D37" s="94" t="s">
+      <c r="D37" s="93" t="s">
         <v>221</v>
       </c>
-      <c r="E37" s="94" t="s">
+      <c r="E37" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F37" s="84"/>
@@ -8137,19 +8133,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="38" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="125"/>
-      <c r="B38" s="94">
+    <row r="38" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="124"/>
+      <c r="B38" s="93">
         <f t="shared" si="2"/>
         <v>36</v>
       </c>
-      <c r="C38" s="101" t="s">
+      <c r="C38" s="100" t="s">
         <v>153</v>
       </c>
-      <c r="D38" s="94" t="s">
+      <c r="D38" s="93" t="s">
         <v>221</v>
       </c>
-      <c r="E38" s="94" t="s">
+      <c r="E38" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F38" s="84"/>
@@ -8185,19 +8181,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:21" ht="18.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="125"/>
-      <c r="B39" s="94">
+    <row r="39" spans="1:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="124"/>
+      <c r="B39" s="93">
         <f t="shared" si="2"/>
         <v>37</v>
       </c>
-      <c r="C39" s="101" t="s">
+      <c r="C39" s="100" t="s">
         <v>154</v>
       </c>
-      <c r="D39" s="94" t="s">
+      <c r="D39" s="93" t="s">
         <v>222</v>
       </c>
-      <c r="E39" s="94" t="s">
+      <c r="E39" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F39" s="84"/>
@@ -8237,19 +8233,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="125"/>
-      <c r="B40" s="94">
+    <row r="40" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="124"/>
+      <c r="B40" s="93">
         <f t="shared" si="2"/>
         <v>38</v>
       </c>
-      <c r="C40" s="101" t="s">
+      <c r="C40" s="100" t="s">
         <v>155</v>
       </c>
-      <c r="D40" s="94" t="s">
+      <c r="D40" s="93" t="s">
         <v>216</v>
       </c>
-      <c r="E40" s="94" t="s">
+      <c r="E40" s="93" t="s">
         <v>183</v>
       </c>
       <c r="F40" s="84"/>
@@ -8285,19 +8281,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="41" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="125"/>
-      <c r="B41" s="94">
+    <row r="41" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="124"/>
+      <c r="B41" s="93">
         <f t="shared" si="2"/>
         <v>39</v>
       </c>
-      <c r="C41" s="101" t="s">
+      <c r="C41" s="100" t="s">
         <v>156</v>
       </c>
-      <c r="D41" s="94" t="s">
+      <c r="D41" s="93" t="s">
         <v>223</v>
       </c>
-      <c r="E41" s="94" t="s">
+      <c r="E41" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F41" s="84"/>
@@ -8333,19 +8329,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="42" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="125"/>
-      <c r="B42" s="94">
+    <row r="42" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="124"/>
+      <c r="B42" s="93">
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="C42" s="101" t="s">
+      <c r="C42" s="100" t="s">
         <v>157</v>
       </c>
-      <c r="D42" s="94" t="s">
+      <c r="D42" s="93" t="s">
         <v>222</v>
       </c>
-      <c r="E42" s="94" t="s">
+      <c r="E42" s="93" t="s">
         <v>181</v>
       </c>
       <c r="F42" s="84"/>
@@ -8383,19 +8379,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="125"/>
-      <c r="B43" s="94">
+    <row r="43" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="124"/>
+      <c r="B43" s="93">
         <f t="shared" si="2"/>
         <v>41</v>
       </c>
-      <c r="C43" s="101" t="s">
+      <c r="C43" s="100" t="s">
         <v>158</v>
       </c>
-      <c r="D43" s="94" t="s">
+      <c r="D43" s="93" t="s">
         <v>215</v>
       </c>
-      <c r="E43" s="94" t="s">
+      <c r="E43" s="93" t="s">
         <v>159</v>
       </c>
       <c r="F43" s="84"/>
@@ -8431,19 +8427,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="44" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="125"/>
-      <c r="B44" s="94">
+    <row r="44" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="124"/>
+      <c r="B44" s="93">
         <f t="shared" si="2"/>
         <v>42</v>
       </c>
-      <c r="C44" s="101" t="s">
+      <c r="C44" s="100" t="s">
         <v>160</v>
       </c>
-      <c r="D44" s="94" t="s">
+      <c r="D44" s="93" t="s">
         <v>224</v>
       </c>
-      <c r="E44" s="94" t="s">
+      <c r="E44" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F44" s="84"/>
@@ -8479,19 +8475,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="45" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="125"/>
-      <c r="B45" s="94">
+    <row r="45" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="124"/>
+      <c r="B45" s="93">
         <f t="shared" si="2"/>
         <v>43</v>
       </c>
-      <c r="C45" s="101" t="s">
+      <c r="C45" s="100" t="s">
         <v>161</v>
       </c>
-      <c r="D45" s="94" t="s">
+      <c r="D45" s="93" t="s">
         <v>225</v>
       </c>
-      <c r="E45" s="94" t="s">
+      <c r="E45" s="93" t="s">
         <v>185</v>
       </c>
       <c r="F45" s="84"/>
@@ -8527,19 +8523,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="46" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="125"/>
-      <c r="B46" s="94">
+    <row r="46" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="124"/>
+      <c r="B46" s="93">
         <f t="shared" si="2"/>
         <v>44</v>
       </c>
-      <c r="C46" s="101" t="s">
+      <c r="C46" s="100" t="s">
         <v>162</v>
       </c>
-      <c r="D46" s="94" t="s">
+      <c r="D46" s="93" t="s">
         <v>221</v>
       </c>
-      <c r="E46" s="94" t="s">
+      <c r="E46" s="93" t="s">
         <v>186</v>
       </c>
       <c r="F46" s="84"/>
@@ -8575,19 +8571,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="47" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="125"/>
-      <c r="B47" s="94">
+    <row r="47" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="124"/>
+      <c r="B47" s="93">
         <f t="shared" si="2"/>
         <v>45</v>
       </c>
-      <c r="C47" s="101" t="s">
+      <c r="C47" s="100" t="s">
         <v>163</v>
       </c>
-      <c r="D47" s="94" t="s">
+      <c r="D47" s="93" t="s">
         <v>226</v>
       </c>
-      <c r="E47" s="94" t="s">
+      <c r="E47" s="93" t="s">
         <v>186</v>
       </c>
       <c r="F47" s="84"/>
@@ -8625,19 +8621,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="48" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="125"/>
-      <c r="B48" s="94">
+    <row r="48" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="124"/>
+      <c r="B48" s="93">
         <f t="shared" si="2"/>
         <v>46</v>
       </c>
-      <c r="C48" s="101" t="s">
+      <c r="C48" s="100" t="s">
         <v>164</v>
       </c>
-      <c r="D48" s="94" t="s">
+      <c r="D48" s="93" t="s">
         <v>226</v>
       </c>
-      <c r="E48" s="94" t="s">
+      <c r="E48" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F48" s="84"/>
@@ -8677,19 +8673,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="49" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="125"/>
-      <c r="B49" s="94">
+    <row r="49" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="124"/>
+      <c r="B49" s="93">
         <f t="shared" si="2"/>
         <v>47</v>
       </c>
-      <c r="C49" s="101" t="s">
+      <c r="C49" s="100" t="s">
         <v>165</v>
       </c>
-      <c r="D49" s="94" t="s">
-        <v>227</v>
-      </c>
-      <c r="E49" s="94" t="s">
+      <c r="D49" s="93" t="s">
+        <v>209</v>
+      </c>
+      <c r="E49" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F49" s="84"/>
@@ -8729,19 +8725,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="125"/>
-      <c r="B50" s="94">
+    <row r="50" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="124"/>
+      <c r="B50" s="93">
         <f t="shared" si="2"/>
         <v>48</v>
       </c>
-      <c r="C50" s="101" t="s">
+      <c r="C50" s="100" t="s">
         <v>166</v>
       </c>
-      <c r="D50" s="94" t="s">
-        <v>227</v>
-      </c>
-      <c r="E50" s="94" t="s">
+      <c r="D50" s="93" t="s">
+        <v>209</v>
+      </c>
+      <c r="E50" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F50" s="84"/>
@@ -8779,19 +8775,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="51" spans="1:21" ht="18.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="125"/>
-      <c r="B51" s="94">
+    <row r="51" spans="1:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="124"/>
+      <c r="B51" s="93">
         <f t="shared" si="2"/>
         <v>49</v>
       </c>
-      <c r="C51" s="101" t="s">
+      <c r="C51" s="100" t="s">
         <v>167</v>
       </c>
-      <c r="D51" s="94" t="s">
-        <v>228</v>
-      </c>
-      <c r="E51" s="94" t="s">
+      <c r="D51" s="93" t="s">
+        <v>227</v>
+      </c>
+      <c r="E51" s="93" t="s">
         <v>187</v>
       </c>
       <c r="F51" s="84"/>
@@ -8829,19 +8825,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="52" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="125"/>
-      <c r="B52" s="94">
+    <row r="52" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="124"/>
+      <c r="B52" s="93">
         <f t="shared" si="2"/>
         <v>50</v>
       </c>
-      <c r="C52" s="101" t="s">
+      <c r="C52" s="100" t="s">
         <v>168</v>
       </c>
-      <c r="D52" s="94" t="s">
-        <v>229</v>
-      </c>
-      <c r="E52" s="94" t="s">
+      <c r="D52" s="93" t="s">
+        <v>228</v>
+      </c>
+      <c r="E52" s="93" t="s">
         <v>184</v>
       </c>
       <c r="F52" s="84"/>
@@ -8879,19 +8875,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="125"/>
-      <c r="B53" s="94">
+    <row r="53" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="124"/>
+      <c r="B53" s="93">
         <f t="shared" si="2"/>
         <v>51</v>
       </c>
-      <c r="C53" s="101" t="s">
+      <c r="C53" s="100" t="s">
         <v>169</v>
       </c>
-      <c r="D53" s="94" t="s">
+      <c r="D53" s="93" t="s">
         <v>199</v>
       </c>
-      <c r="E53" s="94" t="s">
+      <c r="E53" s="93" t="s">
         <v>138</v>
       </c>
       <c r="F53" s="84"/>
@@ -8927,19 +8923,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="54" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="125"/>
-      <c r="B54" s="94">
+    <row r="54" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="124"/>
+      <c r="B54" s="93">
         <f t="shared" si="2"/>
         <v>52</v>
       </c>
-      <c r="C54" s="101" t="s">
+      <c r="C54" s="100" t="s">
         <v>170</v>
       </c>
-      <c r="D54" s="94" t="s">
-        <v>230</v>
-      </c>
-      <c r="E54" s="94" t="s">
+      <c r="D54" s="93" t="s">
+        <v>229</v>
+      </c>
+      <c r="E54" s="93" t="s">
         <v>182</v>
       </c>
       <c r="F54" s="84"/>
@@ -8977,21 +8973,21 @@
         <v>116</v>
       </c>
     </row>
-    <row r="55" spans="1:21" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="117" t="s">
+    <row r="55" spans="1:21" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="116" t="s">
         <v>171</v>
       </c>
-      <c r="B55" s="95">
+      <c r="B55" s="94">
         <f>B54+1</f>
         <v>53</v>
       </c>
-      <c r="C55" s="102" t="s">
+      <c r="C55" s="101" t="s">
         <v>172</v>
       </c>
-      <c r="D55" s="95" t="s">
+      <c r="D55" s="94" t="s">
         <v>217</v>
       </c>
-      <c r="E55" s="95" t="s">
+      <c r="E55" s="94" t="s">
         <v>138</v>
       </c>
       <c r="F55" s="75"/>
@@ -9031,19 +9027,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="117"/>
-      <c r="B56" s="95">
+    <row r="56" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="116"/>
+      <c r="B56" s="94">
         <f t="shared" ref="B56:B63" si="3">B55+1</f>
         <v>54</v>
       </c>
-      <c r="C56" s="102" t="s">
+      <c r="C56" s="101" t="s">
         <v>173</v>
       </c>
-      <c r="D56" s="95" t="s">
-        <v>231</v>
-      </c>
-      <c r="E56" s="95" t="s">
+      <c r="D56" s="94" t="s">
+        <v>230</v>
+      </c>
+      <c r="E56" s="94" t="s">
         <v>188</v>
       </c>
       <c r="F56" s="75"/>
@@ -9083,19 +9079,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:21" ht="18.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="117"/>
-      <c r="B57" s="95">
+    <row r="57" spans="1:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="116"/>
+      <c r="B57" s="94">
         <f t="shared" si="3"/>
         <v>55</v>
       </c>
-      <c r="C57" s="102" t="s">
+      <c r="C57" s="101" t="s">
         <v>174</v>
       </c>
-      <c r="D57" s="95" t="s">
-        <v>232</v>
-      </c>
-      <c r="E57" s="95" t="s">
+      <c r="D57" s="94" t="s">
+        <v>231</v>
+      </c>
+      <c r="E57" s="94" t="s">
         <v>182</v>
       </c>
       <c r="F57" s="75"/>
@@ -9131,19 +9127,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="58" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="117"/>
-      <c r="B58" s="95">
+    <row r="58" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="116"/>
+      <c r="B58" s="94">
         <f t="shared" si="3"/>
         <v>56</v>
       </c>
-      <c r="C58" s="102" t="s">
+      <c r="C58" s="101" t="s">
         <v>175</v>
       </c>
-      <c r="D58" s="95" t="s">
-        <v>233</v>
-      </c>
-      <c r="E58" s="95" t="s">
+      <c r="D58" s="94" t="s">
+        <v>232</v>
+      </c>
+      <c r="E58" s="94" t="s">
         <v>159</v>
       </c>
       <c r="F58" s="75"/>
@@ -9179,19 +9175,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="59" spans="1:21" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="117"/>
-      <c r="B59" s="95">
+    <row r="59" spans="1:21" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="116"/>
+      <c r="B59" s="94">
         <f t="shared" si="3"/>
         <v>57</v>
       </c>
-      <c r="C59" s="102" t="s">
+      <c r="C59" s="101" t="s">
         <v>176</v>
       </c>
-      <c r="D59" s="95" t="s">
-        <v>234</v>
-      </c>
-      <c r="E59" s="95" t="s">
+      <c r="D59" s="94" t="s">
+        <v>233</v>
+      </c>
+      <c r="E59" s="94" t="s">
         <v>159</v>
       </c>
       <c r="F59" s="75"/>
@@ -9227,19 +9223,19 @@
         <v>116</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="117"/>
-      <c r="B60" s="95">
+    <row r="60" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="116"/>
+      <c r="B60" s="94">
         <f t="shared" si="3"/>
         <v>58</v>
       </c>
-      <c r="C60" s="102" t="s">
+      <c r="C60" s="101" t="s">
         <v>177</v>
       </c>
-      <c r="D60" s="95" t="s">
+      <c r="D60" s="94" t="s">
         <v>211</v>
       </c>
-      <c r="E60" s="95" t="s">
+      <c r="E60" s="94" t="s">
         <v>182</v>
       </c>
       <c r="F60" s="75"/>
@@ -9275,19 +9271,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="117"/>
-      <c r="B61" s="95">
+    <row r="61" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="116"/>
+      <c r="B61" s="94">
         <f t="shared" si="3"/>
         <v>59</v>
       </c>
-      <c r="C61" s="102" t="s">
+      <c r="C61" s="101" t="s">
         <v>178</v>
       </c>
-      <c r="D61" s="95" t="s">
-        <v>235</v>
-      </c>
-      <c r="E61" s="95" t="s">
+      <c r="D61" s="94" t="s">
+        <v>234</v>
+      </c>
+      <c r="E61" s="94" t="s">
         <v>182</v>
       </c>
       <c r="F61" s="75"/>
@@ -9325,19 +9321,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="117"/>
-      <c r="B62" s="95">
+    <row r="62" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="116"/>
+      <c r="B62" s="94">
         <f t="shared" si="3"/>
         <v>60</v>
       </c>
-      <c r="C62" s="102" t="s">
+      <c r="C62" s="101" t="s">
         <v>179</v>
       </c>
-      <c r="D62" s="95" t="s">
-        <v>236</v>
-      </c>
-      <c r="E62" s="95" t="s">
+      <c r="D62" s="94" t="s">
+        <v>235</v>
+      </c>
+      <c r="E62" s="94" t="s">
         <v>182</v>
       </c>
       <c r="F62" s="75"/>
@@ -9373,19 +9369,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="117"/>
-      <c r="B63" s="95">
+    <row r="63" spans="1:21" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="116"/>
+      <c r="B63" s="94">
         <f t="shared" si="3"/>
         <v>61</v>
       </c>
-      <c r="C63" s="102" t="s">
+      <c r="C63" s="101" t="s">
         <v>180</v>
       </c>
-      <c r="D63" s="95" t="s">
-        <v>237</v>
-      </c>
-      <c r="E63" s="95" t="s">
+      <c r="D63" s="94" t="s">
+        <v>236</v>
+      </c>
+      <c r="E63" s="94" t="s">
         <v>189</v>
       </c>
       <c r="F63" s="75"/>
@@ -9421,12 +9417,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B64" s="76"/>
       <c r="C64" s="77"/>
-      <c r="D64" s="96"/>
+      <c r="D64" s="95"/>
       <c r="E64" s="76"/>
-      <c r="F64" s="96"/>
+      <c r="F64" s="95"/>
       <c r="G64" s="76"/>
       <c r="H64" s="76"/>
       <c r="I64" s="76"/>
@@ -9441,13 +9437,13 @@
       <c r="S64" s="80"/>
       <c r="T64" s="80"/>
     </row>
-    <row r="65" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="81"/>
       <c r="B65" s="76"/>
       <c r="C65" s="77"/>
-      <c r="D65" s="96"/>
+      <c r="D65" s="95"/>
       <c r="E65" s="76"/>
-      <c r="F65" s="96"/>
+      <c r="F65" s="95"/>
       <c r="G65" s="76"/>
       <c r="H65" s="76"/>
       <c r="I65" s="76"/>
@@ -9464,32 +9460,32 @@
       <c r="T65" s="82"/>
       <c r="U65" s="72"/>
     </row>
-    <row r="66" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A66" s="81"/>
     </row>
-    <row r="67" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A67" s="81"/>
     </row>
-    <row r="68" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A68" s="81"/>
     </row>
-    <row r="69" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A69" s="81"/>
     </row>
-    <row r="70" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A70" s="81"/>
     </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A71" s="81"/>
     </row>
-    <row r="72" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A72" s="81"/>
     </row>
-    <row r="73" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A73" s="81"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="0597I8HImh4F9z/A7w2mUw0K3eEHHDpvAvp6XylF25KORn49mFD8b1+7s95xaT6kKXMThkQEMn4QocudbWAIvw==" saltValue="LubhmbeNnYcArVpvOt52lg==" spinCount="100000" sheet="1" autoFilter="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="Xu7tST2UyvUflGvNaCzhTJ1V/y6E16/9vZyQRivUkrXKRVJ24TctmG59kj03lr2+iemhQQaIQcw08zMzny4LZQ==" saltValue="BkS29aj2Vm//vLh273lc/Q==" spinCount="100000" sheet="1" autoFilter="0"/>
   <autoFilter ref="A2:U65" xr:uid="{40CE4B58-4DDE-4FFB-AF5D-92EC82F1F313}"/>
   <mergeCells count="6">
     <mergeCell ref="A55:A63"/>
@@ -9499,15 +9495,15 @@
     <mergeCell ref="A22:A27"/>
     <mergeCell ref="A28:A54"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="whole" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L7 L3:L4 M61 L9 M10 M14 M16 M21 M23:M26 L23 L26:L27 L30 M31 M33:M36 L37 L39:M39 L42 M47:M50 L48:L49 L51 M52 M54:M56 L55:L56 M3 N3 O3 O4 N4 N5:N18 O15 P14 P18 O18 N19:N22 O21:O27 P23:P25 Q56 P28:Q29 Q30:Q37 O37:P38 P39 O40:O41 P46 Q25 Q24 T60:T63 S28:S30 R34:S34 R37:S39 S40:S41 R42:S50 T44 R51:S52 S53:S54 R54 T55:T59 R25:R30 R24 U22:U23 U26 U38:U39 U42 U55:U56 U60:U63" xr:uid="{8D995782-9C34-4E27-8832-B7B40AFB5170}">
+  <dataValidations count="1">
+    <dataValidation type="whole" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L7 L3:L4 M61 L9 M10 M14 M16 M21 M23:M26 L23 L26:L27 L30 M31 M33:M36 L37 L39:M39 L42 M47:M50 L48:L49 L51 M52 M54:M56 L55:L56 M3 O3:O4 O15 P14 O18:P18 N3:N22 O21:O27 P23:P25 Q56 P28:Q29 Q30:Q37 O37:P38 P39 O40:O41 P46 Q24:Q25 S28:S30 R34:S34 R37:S39 S40:S41 T44 R42:S52 S53:S54 R54 T55:T59 R24:R30 U22:U23 U26 U38:U39 U42 U55:U56 T60:U63" xr:uid="{8D995782-9C34-4E27-8832-B7B40AFB5170}">
       <formula1>1</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="N1:U1" r:id="rId1" display="ONS Quality Standard for Analysis Phases (mapping to QQ)" xr:uid="{738D2B97-F3BD-4FDE-8272-ABCE9901DFFB}"/>
     <hyperlink ref="L2" r:id="rId2" display="Analysis Function Guidance (Quality Q and Red F)" xr:uid="{C326AE48-58B3-4656-A65A-B2EA8649E904}"/>
-    <hyperlink ref="M2" r:id="rId3" display="OSR Guidance" xr:uid="{5BA16752-6848-4CA7-8FA9-C75C10775F25}"/>
+    <hyperlink ref="M2" r:id="rId3" xr:uid="{5BA16752-6848-4CA7-8FA9-C75C10775F25}"/>
     <hyperlink ref="D2" r:id="rId4" xr:uid="{DC07AB57-F3D3-4D54-8EDC-B61894755AC9}"/>
     <hyperlink ref="A2" r:id="rId5" location="roles" xr:uid="{095F8ED3-C96B-4E3C-ACB9-7B45814E01A1}"/>
     <hyperlink ref="E2" r:id="rId6" location="roles" xr:uid="{03048F9D-EB72-4350-8A41-0769749E87F0}"/>
@@ -9522,12 +9518,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7e1cd103-0302-4a32-9a4b-e115c950d959">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="50b62f6a-6a2d-4510-bfe7-b1a3c00072e4" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9780,20 +9778,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7e1cd103-0302-4a32-9a4b-e115c950d959">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="50b62f6a-6a2d-4510-bfe7-b1a3c00072e4" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26A7238D-7DAD-4EFF-B184-28E2DF4DDCD9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85AF8313-FA00-4D59-B28F-14781BE72D64}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="50b62f6a-6a2d-4510-bfe7-b1a3c00072e4"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="7e1cd103-0302-4a32-9a4b-e115c950d959"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9818,18 +9823,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85AF8313-FA00-4D59-B28F-14781BE72D64}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26A7238D-7DAD-4EFF-B184-28E2DF4DDCD9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="50b62f6a-6a2d-4510-bfe7-b1a3c00072e4"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="7e1cd103-0302-4a32-9a4b-e115c950d959"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>